<commit_message>
Update latest objectives result
</commit_message>
<xml_diff>
--- a/latest/objectives_latest.xlsx
+++ b/latest/objectives_latest.xlsx
@@ -611,6 +611,7 @@
         <is>
           <t>Saudi Arabia: Goal 10회
 Germany: 2경기 각 Goal 1회
+TOTS: Outside Box Goal 5회
 CONMEBOL Libertadores: 5경기 각 Goal 1회
 Frauen-Bundesliga: 2경기 각 Goal 1회</t>
         </is>
@@ -625,6 +626,7 @@
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Midfielder: Assist 4회
+TOTS: 1경기 각 Through Ball Assist 1회
 Defender: Assist 4회</t>
         </is>
       </c>
@@ -637,9 +639,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>TOTS: 1경기 각각 Through Ball Assist 1회 이상
-TOTS: Outside Box Goal 5회
-Clean Sheet 5
+          <t>Clean Sheet 5
 Clean Sheet 4</t>
         </is>
       </c>
@@ -13932,7 +13932,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Weekly Objectives Complete weekly Objectives to earn SP! 250 SP Expires in 17 hours 1,250 total 5 Objectives 88% 12%</t>
+          <t>Weekly Objectives Complete weekly Objectives to earn SP! 250 SP Expires in 15 hours 1,250 total 5 Objectives 88% 12%</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -13976,7 +13976,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Season 7 Weekly Play 2 Complete 3 out of the 5 challenges to earn SP! 300 SP Expires in 17 hours 1,050 total 3 of 5 Objectives 85% 15%</t>
+          <t>Season 7 Weekly Play 2 Complete 3 out of the 5 challenges to earn SP! 300 SP Expires in 15 hours 1,050 total 3 of 5 Objectives 85% 15%</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Daily Objectives Play, complete, and earn SP from the daily Objective every 24 hours! 50 SP Expires in 17 hours 150 total 2 Objectives 93% 7%</t>
+          <t>Daily Objectives Play, complete, and earn SP from the daily Objective every 24 hours! 50 SP Expires in 15 hours 150 total 2 Objectives 93% 7%</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -14572,7 +14572,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Clean Sheet, Outside Box Goal, Finesse Goal 등 Goal/Assist 외 특수 수행조건을 표시합니다. 특수조건 파싱이 애매하면 원문을 그대로 표시합니다.</t>
+          <t>Clean Sheet 등 Goal/Assist가 아닌 특수 수행조건을 표시합니다. Outside Box Goal, Through Ball Assist처럼 골/어시 계열은 Goals/Assists로 분류합니다.</t>
         </is>
       </c>
     </row>
@@ -15168,12 +15168,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TOTS: 1경기 각 Through Ball Assist 1회</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>TOTS: 1경기 각각 Through Ball Assist 1회 이상</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -15219,7 +15219,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TOTS: Outside Box Goal 5회</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -15229,7 +15229,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>TOTS: Outside Box Goal 5회</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -18173,12 +18173,12 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TOTS: 1경기 각 Through Ball Assist 1회</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>TOTS: 1경기 각각 Through Ball Assist 1회 이상</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TOTS: Outside Box Goal 5회</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -18259,7 +18259,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>TOTS: Outside Box Goal 5회</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -21285,6 +21285,7 @@
         <is>
           <t>Saudi Arabia: Goal 10회
 Germany: 2경기 각 Goal 1회
+TOTS: Outside Box Goal 5회
 CONMEBOL Libertadores: 5경기 각 Goal 1회
 Frauen-Bundesliga: 2경기 각 Goal 1회</t>
         </is>
@@ -21292,14 +21293,13 @@
       <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Midfielder: Assist 4회
+TOTS: 1경기 각 Through Ball Assist 1회
 Defender: Assist 4회</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>TOTS: 1경기 각각 Through Ball Assist 1회 이상
-TOTS: Outside Box Goal 5회
-Clean Sheet 5
+          <t>Clean Sheet 5
 Clean Sheet 4</t>
         </is>
       </c>
@@ -21950,6 +21950,7 @@
         <is>
           <t>Saudi Arabia: Goal 10회
 Germany: 2경기 각 Goal 1회
+TOTS: Outside Box Goal 5회
 CONMEBOL Libertadores: 5경기 각 Goal 1회
 Frauen-Bundesliga: 2경기 각 Goal 1회</t>
         </is>
@@ -21957,14 +21958,13 @@
       <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Midfielder: Assist 4회
+TOTS: 1경기 각 Through Ball Assist 1회
 Defender: Assist 4회</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>TOTS: 1경기 각각 Through Ball Assist 1회 이상
-TOTS: Outside Box Goal 5회
-Clean Sheet 5
+          <t>Clean Sheet 5
 Clean Sheet 4</t>
         </is>
       </c>
@@ -28265,12 +28265,12 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TOTS: 1경기 각 Through Ball Assist 1회</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>TOTS: 1경기 각각 Through Ball Assist 1회 이상</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -28341,7 +28341,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TOTS: Outside Box Goal 5회</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -28351,7 +28351,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>TOTS: Outside Box Goal 5회</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -35624,6 +35624,7 @@
         <is>
           <t>Saudi Arabia: Goal 10회
 Germany: 2경기 각 Goal 1회
+TOTS: Outside Box Goal 5회
 CONMEBOL Libertadores: 5경기 각 Goal 1회
 Frauen-Bundesliga: 2경기 각 Goal 1회
 Any: 60경기 각 Goal 1회
@@ -35634,15 +35635,14 @@
       <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Midfielder: Assist 4회
+TOTS: 1경기 각 Through Ball Assist 1회
 Defender: Assist 4회
 Any: 35경기 각 Assist 1회</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>TOTS: 1경기 각각 Through Ball Assist 1회 이상
-TOTS: Outside Box Goal 5회
-Clean Sheet 5
+          <t>Clean Sheet 5
 Clean Sheet 4
 Clean Sheet 15
 Clean Sheet 20

</xml_diff>

<commit_message>
Update latest objectives result and summary json
</commit_message>
<xml_diff>
--- a/latest/objectives_latest.xlsx
+++ b/latest/objectives_latest.xlsx
@@ -4422,17 +4422,17 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -4509,17 +4509,17 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -4596,17 +4596,17 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -4683,17 +4683,17 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -4770,17 +4770,17 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -10153,17 +10153,17 @@
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="F87" s="8" t="inlineStr">
@@ -10244,17 +10244,17 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="F88" s="8" t="inlineStr">
@@ -10335,17 +10335,17 @@
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="F89" s="8" t="inlineStr">
@@ -10426,17 +10426,17 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="F90" s="8" t="inlineStr">
@@ -10517,17 +10517,17 @@
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="F91" s="8" t="inlineStr">
@@ -10608,17 +10608,17 @@
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="D92" s="8" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="F92" s="8" t="inlineStr">
@@ -19595,7 +19595,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>French TOTS Flash Rush Join the "French TOTS" Flash Rush event and complete 4 of 5 challenges to earn Pack rewards, an Evolution and SP! All rewards are untradeable. 10X 82+ Rare Gold Players Pack Expires in 16 hours 100 total 4 of 5 Objectives 56% 44%</t>
+          <t>French TOTS Flash Rush Join the "French TOTS" Flash Rush event and complete 4 of 5 challenges to earn Pack rewards, an Evolution and SP! All rewards are untradeable. 10X 82+ Rare Gold Players Pack Expires in 15 hours 100 total 4 of 5 Objectives 56% 44%</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -19605,17 +19605,17 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
     </row>
@@ -20076,7 +20076,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Weekly Rush Points Complete Rush Bonuses alongside your teammates to earn Rush Points! 88+ Rare Gold Player Pack Expires in 17 hours 5 Objectives 18% 82%</t>
+          <t>Weekly Rush Points Complete Rush Bonuses alongside your teammates to earn Rush Points! 88+ Rare Gold Player Pack Expires in 16 hours 5 Objectives 18% 82%</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -20086,17 +20086,17 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
     </row>
@@ -24857,17 +24857,17 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -24954,17 +24954,17 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -25051,17 +25051,17 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -25148,17 +25148,17 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -25245,17 +25245,17 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -29703,17 +29703,17 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -29800,17 +29800,17 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -29897,17 +29897,17 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -29994,17 +29994,17 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -30091,17 +30091,17 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -30188,17 +30188,17 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
@@ -39032,17 +39032,17 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -39129,17 +39129,17 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -39226,17 +39226,17 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -39323,17 +39323,17 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -39420,17 +39420,17 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Expires in 16 hours</t>
+          <t>Expires in 15 hours</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>5/12 18:00</t>
+          <t>5/12 17:00</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T18:00+09:00</t>
+          <t>2026-05-12T17:00+09:00</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -45345,17 +45345,17 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -45442,17 +45442,17 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -45539,17 +45539,17 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
@@ -45636,17 +45636,17 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -45733,17 +45733,17 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
@@ -45830,17 +45830,17 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Expires in 17 hours</t>
+          <t>Expires in 16 hours</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>5/12 19:00</t>
+          <t>5/12 18:00</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12T19:00+09:00</t>
+          <t>2026-05-12T18:00+09:00</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update latest objectives xlsx
</commit_message>
<xml_diff>
--- a/latest/objectives_latest.xlsx
+++ b/latest/objectives_latest.xlsx
@@ -27,7 +27,7 @@
     <sheet name="How_To_Read" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SB_Report'!$A$1:$C$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SB_Report'!$A$1:$C$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'SB_Action_Detail'!$A$1:$O$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Combo_Report_Index'!$A$1:$G$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'New_Report_Index'!$A$1:$F$2</definedName>
@@ -39,7 +39,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Seasonal_Mode_Plan'!$A$1:$J$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Mode_Plan_All'!$A$1:$J$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Mission_DB'!$A$1:$S$110</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Condition_DB'!$A$1:$I$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Condition_DB'!$A$1:$I$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Conflict_Check'!$A$1:$E$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Parse_Check'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Collected_URLs'!$A$1:$G$29</definedName>
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -915,7 +915,7 @@
       <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Any: 5경기 각 Finesse Goal 1회</t>
+          <t>4-1-2-1-2 (2) 전술: 5경기 각 Finesse Goal 1회</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -984,7 +984,7 @@
       <c r="A32" s="2" t="inlineStr"/>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Any: 4경기 각 Cross Assist 1회</t>
+          <t>3-4-2-1 전술: 4경기 각 Cross Assist 1회</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -1144,7 +1144,7 @@
       <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>4-1-2-1-2 (2) 전술 사용</t>
+          <t>5-4-1 전술로 5승</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -1157,12 +1157,12 @@
       <c r="A45" s="2" t="inlineStr"/>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>3-4-2-1 전술 사용</t>
+          <t>Denmark 선수 1명 이상 선발하고 10경기 플레이</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Adapt Your Tactics (마감 5/22 02:00)</t>
+          <t>TOTS HM Hjulmand (마감 5/22 02:00)</t>
         </is>
       </c>
     </row>
@@ -1170,12 +1170,12 @@
       <c r="A46" s="2" t="inlineStr"/>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>5-4-1 전술로 5승</t>
+          <t>4경기 각각 1실점 이하</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Adapt Your Tactics (마감 5/22 02:00)</t>
+          <t>TOTS HM Hjulmand (마감 5/22 02:00)</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       <c r="A47" s="2" t="inlineStr"/>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Denmark 선수 1명 이상 선발하고 10경기 플레이</t>
+          <t>Denmark 선수 2명 이상 선발하고 7승</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -1196,12 +1196,12 @@
       <c r="A48" s="2" t="inlineStr"/>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>4경기 각각 1실점 이하</t>
+          <t>라리가 선수 1명 이상 선발하고 2경기 플레이</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>TOTS HM Hjulmand (마감 5/22 02:00)</t>
+          <t>Silver TOTS HM Trio (마감 5/22 02:00)</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1209,12 @@
       <c r="A49" s="2" t="inlineStr"/>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Denmark 선수 2명 이상 선발하고 7승</t>
+          <t>TOTS 카드 1명 이상 선발하고 2승</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>TOTS HM Hjulmand (마감 5/22 02:00)</t>
+          <t>Silver TOTS HM Trio (마감 5/22 02:00)</t>
         </is>
       </c>
     </row>
@@ -1222,12 +1222,12 @@
       <c r="A50" s="2" t="inlineStr"/>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>라리가 선수 1명 이상 선발하고 2경기 플레이</t>
+          <t>미국 선수 1명 이상 선발하고 2경기 플레이</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Silver TOTS HM Trio (마감 5/22 02:00)</t>
+          <t>Silver TOTS HM Sarah Schupansky (마감 5/21 13:00)</t>
         </is>
       </c>
     </row>
@@ -1235,43 +1235,17 @@
       <c r="A51" s="2" t="inlineStr"/>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>TOTS 카드 1명 이상 선발하고 2승</t>
+          <t>미국 선수 1명 이상 선발하고 2승</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Silver TOTS HM Trio (마감 5/22 02:00)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>미국 선수 1명 이상 선발하고 2경기 플레이</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
           <t>Silver TOTS HM Sarah Schupansky (마감 5/21 13:00)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>미국 선수 1명 이상 선발하고 2승</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>Silver TOTS HM Sarah Schupansky (마감 5/21 13:00)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C53"/>
+  <autoFilter ref="A1:C51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2442,7 +2416,7 @@
           <t>LALIGA ST: Goal 10회
 Any: 5경기 각 Goal 1회
 Liga F: Goal 10회
-Any: 5경기 각 Finesse Goal 1회
+4-1-2-1-2 (2) 전술: 5경기 각 Finesse Goal 1회
 Liga F: 2경기 각 Goal 1회
 NWSL: Goal 2회
 Any: 15경기 각 Finesse Goal 1회</t>
@@ -2452,7 +2426,7 @@
         <is>
           <t>Striker: Assist 4회
 Attacker: Assist 4회
-Any: 4경기 각 Cross Assist 1회
+3-4-2-1 전술: 4경기 각 Cross Assist 1회
 midfielder: Assist 4회
 Liga Portugal: 5경기 각 Assist 1회</t>
         </is>
@@ -2464,8 +2438,6 @@
 Spain 선수 1명 이상 선발하고 6경기 플레이
 4-4-2 전술로 5경기 플레이
 5-3-2 전술로 5경기 각각 1실점 이하
-4-1-2-1-2 (2) 전술 사용
-3-4-2-1 전술 사용
 5-4-1 전술로 5승
 Denmark 선수 1명 이상 선발하고 10경기 플레이
 4경기 각각 1실점 이하
@@ -12376,7 +12348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13607,12 +13579,12 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Formation</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>4-1-2-1-2 (2) 전술</t>
         </is>
       </c>
       <c r="F30" s="8" t="n">
@@ -13626,38 +13598,38 @@
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>Any: 5경기 각각 Finesse Goal 1회 이상</t>
+          <t>4-1-2-1-2 (2) 전술: 5경기 각각 Finesse Goal 1회 이상</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>O008-03</t>
+          <t>O008-04</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Other_Action</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
+          <t>Cross Assist</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
           <t>Formation</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Formation</t>
-        </is>
-      </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>4-1-2-1-2 (2)</t>
+          <t>3-4-2-1 전술</t>
         </is>
       </c>
       <c r="F31" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G31" s="8" t="inlineStr"/>
       <c r="H31" s="8" t="inlineStr">
@@ -13667,24 +13639,24 @@
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>4-1-2-1-2 (2) 전술 사용</t>
+          <t>3-4-2-1 전술: 4경기 각각 Cross Assist 1회 이상</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>O008-04</t>
+          <t>O008-05</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Cross Assist</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -13698,24 +13670,24 @@
         </is>
       </c>
       <c r="F32" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G32" s="8" t="inlineStr"/>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>Any: 4경기 각각 Cross Assist 1회 이상</t>
+          <t>Win 5</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>O008-04</t>
+          <t>O008-05</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -13735,52 +13707,52 @@
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>3-4-2-1</t>
+          <t>5-4-1</t>
         </is>
       </c>
       <c r="F33" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G33" s="8" t="inlineStr"/>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>3-4-2-1 전술 사용</t>
+          <t>5-4-1 전술로 5승</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>O008-05</t>
+          <t>O009-01</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="F34" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G34" s="8" t="inlineStr"/>
       <c r="H34" s="8" t="inlineStr">
@@ -13790,38 +13762,38 @@
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>Win 5</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>O008-05</t>
+          <t>O009-01</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Other_Action</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Formation</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Formation</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>5-4-1</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F35" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G35" s="8" t="inlineStr"/>
       <c r="H35" s="8" t="inlineStr">
@@ -13831,24 +13803,24 @@
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>5-4-1 전술로 5승</t>
+          <t>Play 10</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>O009-01</t>
+          <t>O009-02</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Assist</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -13858,11 +13830,11 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>midfielder</t>
         </is>
       </c>
       <c r="F36" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G36" s="8" t="inlineStr"/>
       <c r="H36" s="8" t="inlineStr">
@@ -13872,38 +13844,38 @@
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>midfielder: Assist 4회</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>O009-01</t>
+          <t>O009-03</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>League</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Liga Portugal</t>
         </is>
       </c>
       <c r="F37" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G37" s="8" t="inlineStr"/>
       <c r="H37" s="8" t="inlineStr">
@@ -13913,34 +13885,34 @@
       </c>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>Play 10</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>O009-02</t>
+          <t>O009-03</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Other_Action</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Assist</t>
+          <t>Concede Limit</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>midfielder</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F38" s="8" t="n">
@@ -13949,19 +13921,19 @@
       <c r="G38" s="8" t="inlineStr"/>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>midfielder: Assist 4회</t>
+          <t>4경기 각각 1실점 이하</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>O009-03</t>
+          <t>O009-04</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -13976,16 +13948,16 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>League</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Liga Portugal</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="F39" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39" s="8" t="inlineStr"/>
       <c r="H39" s="8" t="inlineStr">
@@ -14002,17 +13974,17 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>O009-03</t>
+          <t>O009-04</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Other_Action</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Concede Limit</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -14026,89 +13998,89 @@
         </is>
       </c>
       <c r="F40" s="8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G40" s="8" t="inlineStr"/>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>4경기 각각 1실점 이하</t>
+          <t>Win 7</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>O009-04</t>
+          <t>O009-05</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Assist</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>League</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Liga Portugal</t>
         </is>
       </c>
       <c r="F41" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G41" s="8" t="inlineStr"/>
       <c r="H41" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>Liga Portugal: 5경기 각각 Assist 1회 이상</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>O009-04</t>
+          <t>O010-01</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>League</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>LALIGA</t>
         </is>
       </c>
       <c r="F42" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G42" s="8" t="inlineStr"/>
       <c r="H42" s="8" t="inlineStr">
@@ -14118,65 +14090,65 @@
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>Win 7</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>O009-05</t>
+          <t>O010-01</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Assist</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>League</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>Liga Portugal</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F43" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G43" s="8" t="inlineStr"/>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>Liga Portugal: 5경기 각각 Assist 1회 이상</t>
+          <t>Play 2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>O010-01</t>
+          <t>O010-02</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -14186,52 +14158,52 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>LALIGA</t>
+          <t>Liga F</t>
         </is>
       </c>
       <c r="F44" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G44" s="8" t="inlineStr"/>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>Liga F: 2경기 각각 Goal 1회 이상</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>O010-01</t>
+          <t>O010-03</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Rarity/Competition</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>TOTS</t>
         </is>
       </c>
       <c r="F45" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G45" s="8" t="inlineStr"/>
       <c r="H45" s="8" t="inlineStr">
@@ -14241,34 +14213,34 @@
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>Play 2</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>O010-02</t>
+          <t>O010-03</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>League</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>Liga F</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F46" s="8" t="n">
@@ -14277,43 +14249,43 @@
       <c r="G46" s="8" t="inlineStr"/>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>Liga F: 2경기 각각 Goal 1회 이상</t>
+          <t>Win 2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>O010-03</t>
+          <t>O011-01</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Rarity/Competition</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>TOTS</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F47" s="8" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G47" s="8" t="inlineStr"/>
       <c r="H47" s="8" t="inlineStr">
@@ -14323,14 +14295,14 @@
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>Play 10</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>O010-03</t>
+          <t>O011-02</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
@@ -14354,7 +14326,7 @@
         </is>
       </c>
       <c r="F48" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G48" s="8" t="inlineStr"/>
       <c r="H48" s="8" t="inlineStr">
@@ -14364,24 +14336,24 @@
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>Win 2</t>
+          <t>Win 5</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>O011-01</t>
+          <t>O011-03</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -14400,19 +14372,19 @@
       <c r="G49" s="8" t="inlineStr"/>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>Play 10</t>
+          <t>Any: 10경기 각각 Goal 1회 이상</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>O011-02</t>
+          <t>O011-04</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
@@ -14436,7 +14408,7 @@
         </is>
       </c>
       <c r="F50" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G50" s="8" t="inlineStr"/>
       <c r="H50" s="8" t="inlineStr">
@@ -14446,14 +14418,14 @@
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>Win 5</t>
+          <t>Win 8</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>O011-03</t>
+          <t>O011-05</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -14463,7 +14435,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>Assist</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -14487,24 +14459,24 @@
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>Any: 10경기 각각 Goal 1회 이상</t>
+          <t>Any: 10경기 각각 Assist 1회 이상</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>O011-04</t>
+          <t>O012-01</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -14518,7 +14490,7 @@
         </is>
       </c>
       <c r="F52" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G52" s="8" t="inlineStr"/>
       <c r="H52" s="8" t="inlineStr">
@@ -14528,14 +14500,14 @@
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>Win 8</t>
+          <t>Play 3</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>O011-05</t>
+          <t>O012-02</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -14545,7 +14517,7 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Assist</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
@@ -14559,34 +14531,34 @@
         </is>
       </c>
       <c r="F53" s="8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G53" s="8" t="inlineStr"/>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>Any: 10경기 각각 Assist 1회 이상</t>
+          <t>Any: Goal 3회</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>O012-01</t>
+          <t>O012-03</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
@@ -14610,24 +14582,24 @@
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>Play 3</t>
+          <t>Win 3</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>O012-02</t>
+          <t>O013-01</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
@@ -14641,7 +14613,7 @@
         </is>
       </c>
       <c r="F55" s="8" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G55" s="8" t="inlineStr"/>
       <c r="H55" s="8" t="inlineStr">
@@ -14651,14 +14623,14 @@
       </c>
       <c r="I55" s="8" t="inlineStr">
         <is>
-          <t>Any: Goal 3회</t>
+          <t>Play 10</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>O012-03</t>
+          <t>O013-02</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
@@ -14682,7 +14654,7 @@
         </is>
       </c>
       <c r="F56" s="8" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G56" s="8" t="inlineStr"/>
       <c r="H56" s="8" t="inlineStr">
@@ -14692,34 +14664,34 @@
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>Win 3</t>
+          <t>Win 10</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>O013-01</t>
+          <t>O013-03</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Dutch</t>
         </is>
       </c>
       <c r="F57" s="8" t="n">
@@ -14733,24 +14705,24 @@
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>Play 10</t>
+          <t>Dutch: Goal 10회</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>O013-02</t>
+          <t>O014-01</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -14764,7 +14736,7 @@
         </is>
       </c>
       <c r="F58" s="8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G58" s="8" t="inlineStr"/>
       <c r="H58" s="8" t="inlineStr">
@@ -14774,14 +14746,14 @@
       </c>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>Win 10</t>
+          <t>Play 3</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>O013-03</t>
+          <t>O014-02</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
@@ -14796,16 +14768,16 @@
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>Dutch</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F59" s="8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G59" s="8" t="inlineStr"/>
       <c r="H59" s="8" t="inlineStr">
@@ -14815,24 +14787,24 @@
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>Dutch: Goal 10회</t>
+          <t>Any: Goal 3회</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>O014-01</t>
+          <t>O014-03</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
@@ -14856,14 +14828,14 @@
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>Play 3</t>
+          <t>Win 3</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>O014-02</t>
+          <t>O015-01</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
@@ -14887,7 +14859,7 @@
         </is>
       </c>
       <c r="F61" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G61" s="8" t="inlineStr"/>
       <c r="H61" s="8" t="inlineStr">
@@ -14897,24 +14869,24 @@
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>Any: Goal 3회</t>
+          <t>Any: Goal 2회</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>O014-03</t>
+          <t>O015-02</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
@@ -14928,7 +14900,7 @@
         </is>
       </c>
       <c r="F62" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G62" s="8" t="inlineStr"/>
       <c r="H62" s="8" t="inlineStr">
@@ -14938,24 +14910,24 @@
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>Win 3</t>
+          <t>Any: Goal 2회</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>O015-01</t>
+          <t>O016-01</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
@@ -14969,7 +14941,7 @@
         </is>
       </c>
       <c r="F63" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G63" s="8" t="inlineStr"/>
       <c r="H63" s="8" t="inlineStr">
@@ -14979,14 +14951,14 @@
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>Any: Goal 2회</t>
+          <t>Play 3</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>O015-02</t>
+          <t>O016-02</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
@@ -15010,7 +14982,7 @@
         </is>
       </c>
       <c r="F64" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G64" s="8" t="inlineStr"/>
       <c r="H64" s="8" t="inlineStr">
@@ -15020,24 +14992,24 @@
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>Any: Goal 2회</t>
+          <t>Any: Goal 3회</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>O016-01</t>
+          <t>O016-03</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
@@ -15061,38 +15033,38 @@
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>Play 3</t>
+          <t>Win 3</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>O016-02</t>
+          <t>O017-01</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Nation</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="F66" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G66" s="8" t="inlineStr"/>
       <c r="H66" s="8" t="inlineStr">
@@ -15102,24 +15074,24 @@
       </c>
       <c r="I66" s="8" t="inlineStr">
         <is>
-          <t>Any: Goal 3회</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>O016-03</t>
+          <t>O017-01</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
@@ -15133,7 +15105,7 @@
         </is>
       </c>
       <c r="F67" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G67" s="8" t="inlineStr"/>
       <c r="H67" s="8" t="inlineStr">
@@ -15143,38 +15115,38 @@
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>Win 3</t>
+          <t>Play 2</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>O017-01</t>
+          <t>O017-02</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Nation</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>NWSL</t>
         </is>
       </c>
       <c r="F68" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G68" s="8" t="inlineStr"/>
       <c r="H68" s="8" t="inlineStr">
@@ -15184,38 +15156,38 @@
       </c>
       <c r="I68" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>NWSL: Goal 2회</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>O017-01</t>
+          <t>O017-03</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Nation</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="F69" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G69" s="8" t="inlineStr"/>
       <c r="H69" s="8" t="inlineStr">
@@ -15225,34 +15197,34 @@
       </c>
       <c r="I69" s="8" t="inlineStr">
         <is>
-          <t>Play 2</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>O017-02</t>
+          <t>O017-03</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>NWSL</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F70" s="8" t="n">
@@ -15266,38 +15238,38 @@
       </c>
       <c r="I70" s="8" t="inlineStr">
         <is>
-          <t>NWSL: Goal 2회</t>
+          <t>Win 2</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>O017-03</t>
+          <t>O018-01</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>Nation</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F71" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G71" s="8" t="inlineStr"/>
       <c r="H71" s="8" t="inlineStr">
@@ -15307,24 +15279,24 @@
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>Play 5</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>O017-03</t>
+          <t>O018-02</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
@@ -15338,7 +15310,7 @@
         </is>
       </c>
       <c r="F72" s="8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G72" s="8" t="inlineStr"/>
       <c r="H72" s="8" t="inlineStr">
@@ -15348,14 +15320,14 @@
       </c>
       <c r="I72" s="8" t="inlineStr">
         <is>
-          <t>Win 2</t>
+          <t>Play 10</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>O018-01</t>
+          <t>O018-03</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
@@ -15379,7 +15351,7 @@
         </is>
       </c>
       <c r="F73" s="8" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G73" s="8" t="inlineStr"/>
       <c r="H73" s="8" t="inlineStr">
@@ -15389,14 +15361,14 @@
       </c>
       <c r="I73" s="8" t="inlineStr">
         <is>
-          <t>Play 5</t>
+          <t>Play 15</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>O018-02</t>
+          <t>O018-04</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
@@ -15420,7 +15392,7 @@
         </is>
       </c>
       <c r="F74" s="8" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G74" s="8" t="inlineStr"/>
       <c r="H74" s="8" t="inlineStr">
@@ -15430,14 +15402,14 @@
       </c>
       <c r="I74" s="8" t="inlineStr">
         <is>
-          <t>Play 10</t>
+          <t>Play 20</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>O018-03</t>
+          <t>O018-05</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
@@ -15461,7 +15433,7 @@
         </is>
       </c>
       <c r="F75" s="8" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G75" s="8" t="inlineStr"/>
       <c r="H75" s="8" t="inlineStr">
@@ -15471,14 +15443,14 @@
       </c>
       <c r="I75" s="8" t="inlineStr">
         <is>
-          <t>Play 15</t>
+          <t>Play 25</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>O018-04</t>
+          <t>O019-01</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
@@ -15502,7 +15474,7 @@
         </is>
       </c>
       <c r="F76" s="8" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G76" s="8" t="inlineStr"/>
       <c r="H76" s="8" t="inlineStr">
@@ -15512,14 +15484,14 @@
       </c>
       <c r="I76" s="8" t="inlineStr">
         <is>
-          <t>Play 20</t>
+          <t>Play 5</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>O018-05</t>
+          <t>O019-02</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
@@ -15543,7 +15515,7 @@
         </is>
       </c>
       <c r="F77" s="8" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G77" s="8" t="inlineStr"/>
       <c r="H77" s="8" t="inlineStr">
@@ -15553,14 +15525,14 @@
       </c>
       <c r="I77" s="8" t="inlineStr">
         <is>
-          <t>Play 25</t>
+          <t>Play 5</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>O019-01</t>
+          <t>O019-03</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
@@ -15601,7 +15573,7 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>O019-02</t>
+          <t>O019-04</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
@@ -15642,7 +15614,7 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>O019-03</t>
+          <t>O019-05</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
@@ -15683,7 +15655,7 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>O019-04</t>
+          <t>O019-06</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
@@ -15724,7 +15696,7 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>O019-05</t>
+          <t>O019-07</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
@@ -15765,7 +15737,7 @@
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>O019-06</t>
+          <t>O019-08</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
@@ -15806,7 +15778,7 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>O019-07</t>
+          <t>O019-09</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
@@ -15847,7 +15819,7 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>O019-08</t>
+          <t>O019-10</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
@@ -15888,7 +15860,7 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>O019-09</t>
+          <t>O021-01</t>
         </is>
       </c>
       <c r="B86" s="8" t="inlineStr">
@@ -15929,7 +15901,7 @@
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>O019-10</t>
+          <t>O021-02</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
@@ -15970,7 +15942,7 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>O021-01</t>
+          <t>O021-03</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
@@ -16011,7 +15983,7 @@
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>O021-02</t>
+          <t>O021-04</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
@@ -16052,7 +16024,7 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>O021-03</t>
+          <t>O021-05</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
@@ -16093,7 +16065,7 @@
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>O021-04</t>
+          <t>O021-06</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
@@ -16134,7 +16106,7 @@
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t>O021-05</t>
+          <t>O021-07</t>
         </is>
       </c>
       <c r="B92" s="8" t="inlineStr">
@@ -16175,7 +16147,7 @@
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>O021-06</t>
+          <t>O021-08</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
@@ -16216,7 +16188,7 @@
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t>O021-07</t>
+          <t>O022-01</t>
         </is>
       </c>
       <c r="B94" s="8" t="inlineStr">
@@ -16240,7 +16212,7 @@
         </is>
       </c>
       <c r="F94" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G94" s="8" t="inlineStr"/>
       <c r="H94" s="8" t="inlineStr">
@@ -16250,24 +16222,24 @@
       </c>
       <c r="I94" s="8" t="inlineStr">
         <is>
-          <t>Play 5</t>
+          <t>Play 3</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>O021-08</t>
+          <t>O022-02</t>
         </is>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr">
@@ -16281,34 +16253,34 @@
         </is>
       </c>
       <c r="F95" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G95" s="8" t="inlineStr"/>
       <c r="H95" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I95" s="8" t="inlineStr">
         <is>
-          <t>Play 5</t>
+          <t>Any: 3경기 각각 Goal 1회 이상</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t>O022-01</t>
+          <t>O022-03</t>
         </is>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr">
@@ -16332,65 +16304,65 @@
       </c>
       <c r="I96" s="8" t="inlineStr">
         <is>
-          <t>Play 3</t>
+          <t>Any: Goal 3회</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>O022-02</t>
+          <t>O023-01</t>
         </is>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Nation</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="F97" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G97" s="8" t="inlineStr"/>
       <c r="H97" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>Any: 3경기 각각 Goal 1회 이상</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t>O022-03</t>
+          <t>O023-01</t>
         </is>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D98" s="8" t="inlineStr">
@@ -16404,7 +16376,7 @@
         </is>
       </c>
       <c r="F98" s="8" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="G98" s="8" t="inlineStr"/>
       <c r="H98" s="8" t="inlineStr">
@@ -16414,14 +16386,14 @@
       </c>
       <c r="I98" s="8" t="inlineStr">
         <is>
-          <t>Any: Goal 3회</t>
+          <t>Play 40</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>O023-01</t>
+          <t>O023-02</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
@@ -16462,17 +16434,17 @@
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t>O023-01</t>
+          <t>O023-02</t>
         </is>
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D100" s="8" t="inlineStr">
@@ -16486,7 +16458,7 @@
         </is>
       </c>
       <c r="F100" s="8" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G100" s="8" t="inlineStr"/>
       <c r="H100" s="8" t="inlineStr">
@@ -16496,14 +16468,14 @@
       </c>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>Play 40</t>
+          <t>Win 20</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>O023-02</t>
+          <t>O024-01</t>
         </is>
       </c>
       <c r="B101" s="8" t="inlineStr">
@@ -16527,7 +16499,7 @@
         </is>
       </c>
       <c r="F101" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G101" s="8" t="inlineStr"/>
       <c r="H101" s="8" t="inlineStr">
@@ -16544,17 +16516,17 @@
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t>O023-02</t>
+          <t>O024-01</t>
         </is>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Other_Action</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Concede Limit</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr">
@@ -16573,43 +16545,43 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I102" s="8" t="inlineStr">
         <is>
-          <t>Win 20</t>
+          <t>20경기 각각 1실점 이하</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>O024-01</t>
+          <t>O024-02</t>
         </is>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Nation</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F103" s="8" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr">
@@ -16619,24 +16591,24 @@
       </c>
       <c r="I103" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>Win 30</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t>O024-01</t>
+          <t>O025-01</t>
         </is>
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>Other_Action</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Concede Limit</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D104" s="8" t="inlineStr">
@@ -16650,34 +16622,34 @@
         </is>
       </c>
       <c r="F104" s="8" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I104" s="8" t="inlineStr">
         <is>
-          <t>20경기 각각 1실점 이하</t>
+          <t>Play 1</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t>O024-02</t>
+          <t>O025-02</t>
         </is>
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
@@ -16691,7 +16663,7 @@
         </is>
       </c>
       <c r="F105" s="8" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr">
@@ -16701,14 +16673,14 @@
       </c>
       <c r="I105" s="8" t="inlineStr">
         <is>
-          <t>Win 30</t>
+          <t>Play 2</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t>O025-01</t>
+          <t>O025-03</t>
         </is>
       </c>
       <c r="B106" s="8" t="inlineStr">
@@ -16732,7 +16704,7 @@
         </is>
       </c>
       <c r="F106" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G106" s="8" t="inlineStr"/>
       <c r="H106" s="8" t="inlineStr">
@@ -16742,14 +16714,14 @@
       </c>
       <c r="I106" s="8" t="inlineStr">
         <is>
-          <t>Play 1</t>
+          <t>Play 3</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t>O025-02</t>
+          <t>O025-04</t>
         </is>
       </c>
       <c r="B107" s="8" t="inlineStr">
@@ -16773,7 +16745,7 @@
         </is>
       </c>
       <c r="F107" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G107" s="8" t="inlineStr"/>
       <c r="H107" s="8" t="inlineStr">
@@ -16783,14 +16755,14 @@
       </c>
       <c r="I107" s="8" t="inlineStr">
         <is>
-          <t>Play 2</t>
+          <t>Play 4</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t>O025-03</t>
+          <t>O025-05</t>
         </is>
       </c>
       <c r="B108" s="8" t="inlineStr">
@@ -16814,7 +16786,7 @@
         </is>
       </c>
       <c r="F108" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G108" s="8" t="inlineStr"/>
       <c r="H108" s="8" t="inlineStr">
@@ -16824,14 +16796,14 @@
       </c>
       <c r="I108" s="8" t="inlineStr">
         <is>
-          <t>Play 3</t>
+          <t>Play 5</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t>O025-04</t>
+          <t>O025-06</t>
         </is>
       </c>
       <c r="B109" s="8" t="inlineStr">
@@ -16855,7 +16827,7 @@
         </is>
       </c>
       <c r="F109" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G109" s="8" t="inlineStr"/>
       <c r="H109" s="8" t="inlineStr">
@@ -16865,38 +16837,38 @@
       </c>
       <c r="I109" s="8" t="inlineStr">
         <is>
-          <t>Play 4</t>
+          <t>Play 6</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t>O025-05</t>
+          <t>O026-01</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D110" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="F110" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G110" s="8" t="inlineStr"/>
       <c r="H110" s="8" t="inlineStr">
@@ -16906,24 +16878,24 @@
       </c>
       <c r="I110" s="8" t="inlineStr">
         <is>
-          <t>Play 5</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t>O025-06</t>
+          <t>O026-01</t>
         </is>
       </c>
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Performer</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Finesse Goal</t>
         </is>
       </c>
       <c r="D111" s="8" t="inlineStr">
@@ -16937,24 +16909,24 @@
         </is>
       </c>
       <c r="F111" s="8" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="G111" s="8" t="inlineStr"/>
       <c r="H111" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I111" s="8" t="inlineStr">
         <is>
-          <t>Play 6</t>
+          <t>Any: 15경기 각각 Finesse Goal 1회 이상</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t>O026-01</t>
+          <t>O026-02</t>
         </is>
       </c>
       <c r="B112" s="8" t="inlineStr">
@@ -16995,17 +16967,17 @@
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t>O026-01</t>
+          <t>O026-02</t>
         </is>
       </c>
       <c r="B113" s="8" t="inlineStr">
         <is>
-          <t>Performer</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t>Finesse Goal</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D113" s="8" t="inlineStr">
@@ -17019,48 +16991,48 @@
         </is>
       </c>
       <c r="F113" s="8" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G113" s="8" t="inlineStr"/>
       <c r="H113" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I113" s="8" t="inlineStr">
         <is>
-          <t>Any: 15경기 각각 Finesse Goal 1회 이상</t>
+          <t>Win 25</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t>O026-02</t>
+          <t>O027-01</t>
         </is>
       </c>
       <c r="B114" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Clean Sheet</t>
         </is>
       </c>
       <c r="D114" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F114" s="8" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="G114" s="8" t="inlineStr"/>
       <c r="H114" s="8" t="inlineStr">
@@ -17070,38 +17042,38 @@
       </c>
       <c r="I114" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>Clean Sheet 20</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t>O026-02</t>
+          <t>O027-02</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
         <is>
-          <t>Match_Result</t>
+          <t>Squad</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>Starting XI</t>
         </is>
       </c>
       <c r="D115" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Nation</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="F115" s="8" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G115" s="8" t="inlineStr"/>
       <c r="H115" s="8" t="inlineStr">
@@ -17111,14 +17083,14 @@
       </c>
       <c r="I115" s="8" t="inlineStr">
         <is>
-          <t>Win 25</t>
+          <t>선발에 포함</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t>O027-01</t>
+          <t>O027-02</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
@@ -17128,7 +17100,7 @@
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t>Clean Sheet</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D116" s="8" t="inlineStr">
@@ -17142,7 +17114,7 @@
         </is>
       </c>
       <c r="F116" s="8" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G116" s="8" t="inlineStr"/>
       <c r="H116" s="8" t="inlineStr">
@@ -17152,38 +17124,38 @@
       </c>
       <c r="I116" s="8" t="inlineStr">
         <is>
-          <t>Clean Sheet 20</t>
+          <t>Win 35</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t>O027-02</t>
+          <t>O028-01</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Match_Count</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t>Starting XI</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D117" s="8" t="inlineStr">
         <is>
-          <t>Nation</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F117" s="8" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="G117" s="8" t="inlineStr"/>
       <c r="H117" s="8" t="inlineStr">
@@ -17193,14 +17165,14 @@
       </c>
       <c r="I117" s="8" t="inlineStr">
         <is>
-          <t>선발에 포함</t>
+          <t>Play 30</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t>O027-02</t>
+          <t>O028-02</t>
         </is>
       </c>
       <c r="B118" s="8" t="inlineStr">
@@ -17224,7 +17196,7 @@
         </is>
       </c>
       <c r="F118" s="8" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="G118" s="8" t="inlineStr"/>
       <c r="H118" s="8" t="inlineStr">
@@ -17234,24 +17206,24 @@
       </c>
       <c r="I118" s="8" t="inlineStr">
         <is>
-          <t>Win 35</t>
+          <t>Win 10</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t>O028-01</t>
+          <t>O028-03</t>
         </is>
       </c>
       <c r="B119" s="8" t="inlineStr">
         <is>
-          <t>Match_Count</t>
+          <t>Match_Result</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="D119" s="8" t="inlineStr">
@@ -17265,7 +17237,7 @@
         </is>
       </c>
       <c r="F119" s="8" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G119" s="8" t="inlineStr"/>
       <c r="H119" s="8" t="inlineStr">
@@ -17275,14 +17247,14 @@
       </c>
       <c r="I119" s="8" t="inlineStr">
         <is>
-          <t>Play 30</t>
+          <t>Win 20</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
         <is>
-          <t>O028-02</t>
+          <t>O028-04</t>
         </is>
       </c>
       <c r="B120" s="8" t="inlineStr">
@@ -17306,7 +17278,7 @@
         </is>
       </c>
       <c r="F120" s="8" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="G120" s="8" t="inlineStr"/>
       <c r="H120" s="8" t="inlineStr">
@@ -17316,14 +17288,14 @@
       </c>
       <c r="I120" s="8" t="inlineStr">
         <is>
-          <t>Win 10</t>
+          <t>Win 30</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t>O028-03</t>
+          <t>O028-05</t>
         </is>
       </c>
       <c r="B121" s="8" t="inlineStr">
@@ -17347,7 +17319,7 @@
         </is>
       </c>
       <c r="F121" s="8" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G121" s="8" t="inlineStr"/>
       <c r="H121" s="8" t="inlineStr">
@@ -17357,94 +17329,12 @@
       </c>
       <c r="I121" s="8" t="inlineStr">
         <is>
-          <t>Win 20</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="8" t="inlineStr">
-        <is>
-          <t>O028-04</t>
-        </is>
-      </c>
-      <c r="B122" s="8" t="inlineStr">
-        <is>
-          <t>Match_Result</t>
-        </is>
-      </c>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="D122" s="8" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="E122" s="8" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="F122" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="G122" s="8" t="inlineStr"/>
-      <c r="H122" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I122" s="8" t="inlineStr">
-        <is>
-          <t>Win 30</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="8" t="inlineStr">
-        <is>
-          <t>O028-05</t>
-        </is>
-      </c>
-      <c r="B123" s="8" t="inlineStr">
-        <is>
-          <t>Match_Result</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="D123" s="8" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="E123" s="8" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="F123" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="G123" s="8" t="inlineStr"/>
-      <c r="H123" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I123" s="8" t="inlineStr">
-        <is>
           <t>Win 40</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I123"/>
+  <autoFilter ref="A1:I121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17737,7 +17627,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Finesse Goal, Formation</t>
+          <t>Finesse Goal</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -20339,7 +20229,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Any: 5경기 각 Finesse Goal 1회</t>
+          <t>4-1-2-1-2 (2) 전술: 5경기 각 Finesse Goal 1회</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
@@ -20349,7 +20239,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>4-1-2-1-2 (2) 전술 사용</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -20415,12 +20305,12 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Any: 4경기 각 Cross Assist 1회</t>
+          <t>3-4-2-1 전술: 4경기 각 Cross Assist 1회</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>3-4-2-1 전술 사용</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -24127,7 +24017,7 @@
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>Any: 5경기 각 Finesse Goal 1회</t>
+          <t>4-1-2-1-2 (2) 전술: 5경기 각 Finesse Goal 1회</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -24137,7 +24027,7 @@
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>4-1-2-1-2 (2) 전술 사용</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr">
@@ -24233,12 +24123,12 @@
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>Any: 4경기 각 Cross Assist 1회</t>
+          <t>3-4-2-1 전술: 4경기 각 Cross Assist 1회</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>3-4-2-1 전술 사용</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">
@@ -28105,7 +27995,7 @@
           <t>LALIGA ST: Goal 10회
 Any: 5경기 각 Goal 1회
 Liga F: Goal 10회
-Any: 5경기 각 Finesse Goal 1회
+4-1-2-1-2 (2) 전술: 5경기 각 Finesse Goal 1회
 Liga F: 2경기 각 Goal 1회
 NWSL: Goal 2회</t>
         </is>
@@ -28114,7 +28004,7 @@
         <is>
           <t>Striker: Assist 4회
 Attacker: Assist 4회
-Any: 4경기 각 Cross Assist 1회
+3-4-2-1 전술: 4경기 각 Cross Assist 1회
 midfielder: Assist 4회
 Liga Portugal: 5경기 각 Assist 1회</t>
         </is>
@@ -28126,8 +28016,6 @@
 Spain 선수 1명 이상 선발하고 6경기 플레이
 4-4-2 전술로 5경기 플레이
 5-3-2 전술로 5경기 각각 1실점 이하
-4-1-2-1-2 (2) 전술 사용
-3-4-2-1 전술 사용
 5-4-1 전술로 5승
 Denmark 선수 1명 이상 선발하고 10경기 플레이
 4경기 각각 1실점 이하
@@ -28740,7 +28628,7 @@
           <t>LALIGA ST: Goal 10회
 Any: 5경기 각 Goal 1회
 Liga F: Goal 10회
-Any: 5경기 각 Finesse Goal 1회
+4-1-2-1-2 (2) 전술: 5경기 각 Finesse Goal 1회
 Liga F: 2경기 각 Goal 1회
 NWSL: Goal 2회</t>
         </is>
@@ -28749,7 +28637,7 @@
         <is>
           <t>Striker: Assist 4회
 Attacker: Assist 4회
-Any: 4경기 각 Cross Assist 1회
+3-4-2-1 전술: 4경기 각 Cross Assist 1회
 midfielder: Assist 4회
 Liga Portugal: 5경기 각 Assist 1회</t>
         </is>
@@ -28761,8 +28649,6 @@
 Spain 선수 1명 이상 선발하고 6경기 플레이
 4-4-2 전술로 5경기 플레이
 5-3-2 전술로 5경기 각각 1실점 이하
-4-1-2-1-2 (2) 전술 사용
-3-4-2-1 전술 사용
 5-4-1 전술로 5승
 Denmark 선수 1명 이상 선발하고 10경기 플레이
 4경기 각각 1실점 이하
@@ -36343,7 +36229,7 @@
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>Any: 5경기 각 Finesse Goal 1회</t>
+          <t>4-1-2-1-2 (2) 전술: 5경기 각 Finesse Goal 1회</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -36353,7 +36239,7 @@
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>4-1-2-1-2 (2) 전술 사용</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr">
@@ -36449,12 +36335,12 @@
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>Any: 4경기 각 Cross Assist 1회</t>
+          <t>3-4-2-1 전술: 4경기 각 Cross Assist 1회</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>3-4-2-1 전술 사용</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">

</xml_diff>